<commit_message>
Pastelería EN F2 ronda 1: los 15 xlsx y los volcados (gates VERDE 8/0, autotest 20/20, 0 celdas cortadas nuevas)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LzWqvTU1jPmLwXsDXHDGWJ
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/pastry-shop-checklist-templates/01-pastry-kitchen-bakery-case-opening-closing-checklists.xlsx
+++ b/astro-site/public/dl/pastry-shop-checklist-templates/01-pastry-kitchen-bakery-case-opening-closing-checklists.xlsx
@@ -1052,7 +1052,7 @@
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>Take out butter / margarine to temper (20 min before laminating)</t>
+          <t>Take butter / margarine out of the walk-in to bring it to working temperature (20 min before laminating)</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Set up the day's mise en place</t>
+          <t>Set up the day's mise en place; hand sinks stocked with soap and paper towels and kept clear (FDA Food Code 6-301.12)</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t>Sanitize work surfaces and marble benches (sanitizer at label strength, checked with a test strip; FDA Food Code 4-501.114)</t>
+          <t>Sanitize work surfaces and marble benches (sanitizer at label strength, checked with a test strip; FDA Food Code 4-501.114); keep nut flours and seeds in closed, labeled bins</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -2135,12 +2135,12 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>Head pastry chef</t>
+          <t>Shift lead</t>
         </is>
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>6:30 PM</t>
+          <t>8:05 PM</t>
         </is>
       </c>
       <c r="F27" s="14" t="n"/>
@@ -2189,7 +2189,7 @@
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
-          <t>Head pastry chef</t>
+          <t>Shift lead</t>
         </is>
       </c>
       <c r="E29" s="13" t="inlineStr">

</xml_diff>